<commit_message>
Support per-agent monthly targets in the weekly sales report
Layan (ATL) and Chaima are on a reduced AED 20,000/month target instead
of the AED 25,000 default; everyone else stays at 25,000. Team weekly
target recalculates to AED 43,844 (was 46,152 under the flat model).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiEcNy7XAwqHLRjhRBareN
</commit_message>
<xml_diff>
--- a/trackers/reports/WEEKLY_SALES_REPORT_2026-09-12.xlsx
+++ b/trackers/reports/WEEKLY_SALES_REPORT_2026-09-12.xlsx
@@ -523,7 +523,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Week Ending: 12-Sep-2026 (assumed — confirm actual week)   |   Team Lead: Bindhi   |   Per-Agent Weekly Target: AED 5,769 (base AED 25,000/mo ÷ 26 working days × 6)</t>
+          <t>Week Ending: 12-Sep-2026 (assumed — confirm actual week)   |   Team Lead: Bindhi   |   Default Monthly Target: AED 25,000/agent   |   Override: Layan (ATL) AED 20,000/mo, Chaima AED 20,000/mo</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46152</v>
+        <v>43844</v>
       </c>
       <c r="B6" s="5">
         <f>C18</f>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5769</v>
+        <v>4615</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>8600</v>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5769</v>
+        <v>4615</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>8041</v>

</xml_diff>